<commit_message>
feat: added spm-49 and test cases
</commit_message>
<xml_diff>
--- a/docs/test-cases/SPM-49_Test_Cases.xlsx
+++ b/docs/test-cases/SPM-49_Test_Cases.xlsx
@@ -37,8 +37,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="6">
     <font>
@@ -162,7 +163,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -189,6 +190,9 @@
     </xf>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1553,7 +1557,11 @@
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B11" s="3" t="n"/>
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>Coordinator's GET /api/events/EVT-000085/equipment -&gt; HTTP 200. Portable Stage row: quantityReserved=2, status=reserved.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -1561,7 +1569,11 @@
           <t>Pass/Fail/Not Executed/Blocked</t>
         </is>
       </c>
-      <c r="B12" s="3" t="n"/>
+      <c r="B12" s="13" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -1569,7 +1581,11 @@
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B13" s="3" t="n"/>
+      <c r="B13" s="13" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -1577,7 +1593,11 @@
           <t>Executed by</t>
         </is>
       </c>
-      <c r="B14" s="3" t="n"/>
+      <c r="B14" s="13" t="inlineStr">
+        <is>
+          <t>Janelle</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -1585,7 +1605,9 @@
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B15" s="3" t="n"/>
+      <c r="B15" s="15" t="n">
+        <v>46292</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1723,7 +1745,11 @@
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B11" s="3" t="n"/>
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>Partner Lunch BEFORE: chip=available, 4 total − 0 in maintenance − 0 reserved elsewhere = 4 available for these dates. AFTER Product Demo Day reserves 3: chip=partial, 4 total − 0 in maintenance − 3 reserved elsewhere = 1 available for these dates, '2 requested, 1 available.'</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -1731,7 +1757,11 @@
           <t>Pass/Fail/Not Executed/Blocked</t>
         </is>
       </c>
-      <c r="B12" s="3" t="n"/>
+      <c r="B12" s="13" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -1739,7 +1769,11 @@
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B13" s="3" t="n"/>
+      <c r="B13" s="13" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -1747,7 +1781,11 @@
           <t>Executed by</t>
         </is>
       </c>
-      <c r="B14" s="3" t="n"/>
+      <c r="B14" s="13" t="inlineStr">
+        <is>
+          <t>Janelle</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -1755,7 +1793,9 @@
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B15" s="3" t="n"/>
+      <c r="B15" s="15" t="n">
+        <v>46292</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1889,7 +1929,11 @@
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B11" s="3" t="n"/>
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>Board Retreat (2027-04-26), unrelated to Sales Kickoff's reservation: chip=available, 4 total − 0 in maintenance − 0 reserved elsewhere = 4 available for these dates.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -1897,7 +1941,11 @@
           <t>Pass/Fail/Not Executed/Blocked</t>
         </is>
       </c>
-      <c r="B12" s="3" t="n"/>
+      <c r="B12" s="13" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -1905,7 +1953,11 @@
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B13" s="3" t="n"/>
+      <c r="B13" s="13" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -1913,7 +1965,11 @@
           <t>Executed by</t>
         </is>
       </c>
-      <c r="B14" s="3" t="n"/>
+      <c r="B14" s="13" t="inlineStr">
+        <is>
+          <t>Janelle</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -1921,7 +1977,9 @@
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B15" s="3" t="n"/>
+      <c r="B15" s="15" t="n">
+        <v>46292</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2056,7 +2114,11 @@
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B11" s="3" t="n"/>
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>Media Briefing (day after Trade Show's Return Day): chip=partial, 4 total − 0 in maintenance − 3 reserved elsewhere = 1 available for these dates, '2 requested, 1 available.'</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -2064,7 +2126,11 @@
           <t>Pass/Fail/Not Executed/Blocked</t>
         </is>
       </c>
-      <c r="B12" s="3" t="n"/>
+      <c r="B12" s="13" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -2072,7 +2138,11 @@
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B13" s="3" t="n"/>
+      <c r="B13" s="13" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -2080,7 +2150,11 @@
           <t>Executed by</t>
         </is>
       </c>
-      <c r="B14" s="3" t="n"/>
+      <c r="B14" s="13" t="inlineStr">
+        <is>
+          <t>Janelle</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -2088,7 +2162,9 @@
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B15" s="3" t="n"/>
+      <c r="B15" s="15" t="n">
+        <v>46292</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2222,7 +2298,11 @@
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B11" s="3" t="n"/>
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>Wrap Party (two days after Careers Day's Return Day): chip=available, 4 total − 0 in maintenance − 0 reserved elsewhere = 4 available for these dates.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -2230,7 +2310,11 @@
           <t>Pass/Fail/Not Executed/Blocked</t>
         </is>
       </c>
-      <c r="B12" s="3" t="n"/>
+      <c r="B12" s="13" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -2238,7 +2322,11 @@
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B13" s="3" t="n"/>
+      <c r="B13" s="13" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -2246,7 +2334,11 @@
           <t>Executed by</t>
         </is>
       </c>
-      <c r="B14" s="3" t="n"/>
+      <c r="B14" s="13" t="inlineStr">
+        <is>
+          <t>Janelle</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -2254,7 +2346,9 @@
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B15" s="3" t="n"/>
+      <c r="B15" s="15" t="n">
+        <v>46292</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2387,7 +2481,11 @@
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B11" s="3" t="n"/>
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>After Innovation Day reserves 3: Reserved=3, breakdown 4 total − 0 in maintenance − 0 reserved elsewhere = 4 available for these dates (own reservation not counted as held elsewhere).</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -2395,7 +2493,11 @@
           <t>Pass/Fail/Not Executed/Blocked</t>
         </is>
       </c>
-      <c r="B12" s="3" t="n"/>
+      <c r="B12" s="13" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -2403,7 +2505,11 @@
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B13" s="3" t="n"/>
+      <c r="B13" s="13" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -2411,7 +2517,11 @@
           <t>Executed by</t>
         </is>
       </c>
-      <c r="B14" s="3" t="n"/>
+      <c r="B14" s="13" t="inlineStr">
+        <is>
+          <t>Janelle</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -2419,7 +2529,9 @@
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B15" s="3" t="n"/>
+      <c r="B15" s="15" t="n">
+        <v>46292</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2550,7 +2662,11 @@
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B11" s="3" t="n"/>
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>Before attempting: chip=unavailable, 2 total − 0 in maintenance − 2 reserved elsewhere = 0 available for these dates. Reserve attempt -&gt; HTTP 400 {'error': 'Nothing is available for these dates any more.'}.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -2558,7 +2674,11 @@
           <t>Pass/Fail/Not Executed/Blocked</t>
         </is>
       </c>
-      <c r="B12" s="3" t="n"/>
+      <c r="B12" s="13" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -2566,7 +2686,11 @@
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B13" s="3" t="n"/>
+      <c r="B13" s="13" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -2574,7 +2698,11 @@
           <t>Executed by</t>
         </is>
       </c>
-      <c r="B14" s="3" t="n"/>
+      <c r="B14" s="13" t="inlineStr">
+        <is>
+          <t>Janelle</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -2582,7 +2710,9 @@
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B15" s="3" t="n"/>
+      <c r="B15" s="15" t="n">
+        <v>46292</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2715,7 +2845,11 @@
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B11" s="3" t="n"/>
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>Before: chip=partial, 4 total − 0 in maintenance − 3 reserved elsewhere = 1 available for these dates. Reserve -&gt; HTTP 200. After: Reserved=1 (not 2), status=partially_fulfilled.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -2723,7 +2857,11 @@
           <t>Pass/Fail/Not Executed/Blocked</t>
         </is>
       </c>
-      <c r="B12" s="3" t="n"/>
+      <c r="B12" s="13" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -2731,7 +2869,11 @@
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B13" s="3" t="n"/>
+      <c r="B13" s="13" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -2739,7 +2881,11 @@
           <t>Executed by</t>
         </is>
       </c>
-      <c r="B14" s="3" t="n"/>
+      <c r="B14" s="13" t="inlineStr">
+        <is>
+          <t>Janelle</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -2747,7 +2893,9 @@
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B15" s="3" t="n"/>
+      <c r="B15" s="15" t="n">
+        <v>46292</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2880,7 +3028,11 @@
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B11" s="3" t="n"/>
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>Concurrent POST reserve, Pop-up Store (Vikram) -&gt; HTTP 200, Flash Sale (Chloe) -&gt; HTTP 400. Exactly one succeeded: Pop-up Store Reserved=1, Flash Sale Reserved=None.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -2888,7 +3040,11 @@
           <t>Pass/Fail/Not Executed/Blocked</t>
         </is>
       </c>
-      <c r="B12" s="3" t="n"/>
+      <c r="B12" s="13" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -2896,7 +3052,11 @@
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B13" s="3" t="n"/>
+      <c r="B13" s="13" t="inlineStr">
+        <is>
+          <t>Executed as two concurrent API calls, not two browser windows - the same server-side lock is exercised either way; the on-screen refusal message can still be eyeballed once.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -2904,7 +3064,11 @@
           <t>Executed by</t>
         </is>
       </c>
-      <c r="B14" s="3" t="n"/>
+      <c r="B14" s="13" t="inlineStr">
+        <is>
+          <t>Janelle</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -2912,7 +3076,9 @@
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B15" s="3" t="n"/>
+      <c r="B15" s="15" t="n">
+        <v>46292</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3044,7 +3210,11 @@
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B11" s="3" t="n"/>
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>Before: chip=partial, 5 total − 2 in maintenance − 0 reserved elsewhere = 3 available for these dates. After reserving: Reserved=3 (not 4), status=partially_fulfilled.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -3052,7 +3222,11 @@
           <t>Pass/Fail/Not Executed/Blocked</t>
         </is>
       </c>
-      <c r="B12" s="3" t="n"/>
+      <c r="B12" s="13" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -3060,7 +3234,11 @@
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B13" s="3" t="n"/>
+      <c r="B13" s="13" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -3068,7 +3246,11 @@
           <t>Executed by</t>
         </is>
       </c>
-      <c r="B14" s="3" t="n"/>
+      <c r="B14" s="13" t="inlineStr">
+        <is>
+          <t>Janelle</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -3076,7 +3258,9 @@
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B15" s="3" t="n"/>
+      <c r="B15" s="15" t="n">
+        <v>46292</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3331,7 +3515,11 @@
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B11" s="3" t="n"/>
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>Reserve attempt on a Cancelled event -&gt; HTTP 400 {'error': 'This event is cancelled — equipment can no longer be reserved.'}. Reserved stays None.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -3339,7 +3527,11 @@
           <t>Pass/Fail/Not Executed/Blocked</t>
         </is>
       </c>
-      <c r="B12" s="3" t="n"/>
+      <c r="B12" s="13" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -3347,7 +3539,11 @@
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B13" s="3" t="n"/>
+      <c r="B13" s="13" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -3355,7 +3551,11 @@
           <t>Executed by</t>
         </is>
       </c>
-      <c r="B14" s="3" t="n"/>
+      <c r="B14" s="13" t="inlineStr">
+        <is>
+          <t>Janelle</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -3363,7 +3563,9 @@
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B15" s="3" t="n"/>
+      <c r="B15" s="15" t="n">
+        <v>46292</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3499,7 +3701,11 @@
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B11" s="3" t="n"/>
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>Day 1: chip=unavailable, 4 total − 0 in maintenance − 4 reserved elsewhere = 0 available for these dates. Day 2 reserve -&gt; HTTP 200, Reserved=2, status=reserved. Day 1 reserve attempt -&gt; HTTP 400 {'error': 'Nothing is available for these dates any more.'}.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -3507,7 +3713,11 @@
           <t>Pass/Fail/Not Executed/Blocked</t>
         </is>
       </c>
-      <c r="B12" s="3" t="n"/>
+      <c r="B12" s="13" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -3515,7 +3725,11 @@
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B13" s="3" t="n"/>
+      <c r="B13" s="13" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -3523,7 +3737,11 @@
           <t>Executed by</t>
         </is>
       </c>
-      <c r="B14" s="3" t="n"/>
+      <c r="B14" s="13" t="inlineStr">
+        <is>
+          <t>Janelle</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -3531,7 +3749,9 @@
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B15" s="3" t="n"/>
+      <c r="B15" s="15" t="n">
+        <v>46292</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3664,7 +3884,11 @@
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B11" s="3" t="n"/>
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>Logged in as chloe.teo, GET availability -&gt; HTTP 200. Portable Stage line: Reserved=3, status=reserved, 6 total − 0 in maintenance − 0 reserved elsewhere = 6 available for these dates.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -3672,7 +3896,11 @@
           <t>Pass/Fail/Not Executed/Blocked</t>
         </is>
       </c>
-      <c r="B12" s="3" t="n"/>
+      <c r="B12" s="13" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -3680,7 +3908,11 @@
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B13" s="3" t="n"/>
+      <c r="B13" s="13" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -3688,7 +3920,11 @@
           <t>Executed by</t>
         </is>
       </c>
-      <c r="B14" s="3" t="n"/>
+      <c r="B14" s="13" t="inlineStr">
+        <is>
+          <t>Janelle</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -3696,7 +3932,9 @@
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B15" s="3" t="n"/>
+      <c r="B15" s="15" t="n">
+        <v>46292</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3826,7 +4064,11 @@
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B11" s="3" t="n"/>
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>Logged in as the Organiser rachel.ng, GET availability -&gt; HTTP 403 {'error': 'Only Technical Support Staff can check equipment availability'}.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -3834,7 +4076,11 @@
           <t>Pass/Fail/Not Executed/Blocked</t>
         </is>
       </c>
-      <c r="B12" s="3" t="n"/>
+      <c r="B12" s="13" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -3842,7 +4088,11 @@
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B13" s="3" t="n"/>
+      <c r="B13" s="13" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -3850,7 +4100,11 @@
           <t>Executed by</t>
         </is>
       </c>
-      <c r="B14" s="3" t="n"/>
+      <c r="B14" s="13" t="inlineStr">
+        <is>
+          <t>Janelle</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -3858,7 +4112,9 @@
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B15" s="3" t="n"/>
+      <c r="B15" s="15" t="n">
+        <v>46292</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3992,7 +4248,11 @@
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B11" s="3" t="n"/>
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>Reserve call -&gt; HTTP 200. After: Reserved=3, status=reserved, 6 total − 0 in maintenance − 0 reserved elsewhere = 6 available for these dates</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -4000,7 +4260,11 @@
           <t>Pass/Fail/Not Executed/Blocked</t>
         </is>
       </c>
-      <c r="B12" s="3" t="n"/>
+      <c r="B12" s="13" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -4008,7 +4272,11 @@
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B13" s="3" t="n"/>
+      <c r="B13" s="13" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -4016,7 +4284,11 @@
           <t>Executed by</t>
         </is>
       </c>
-      <c r="B14" s="3" t="n"/>
+      <c r="B14" s="13" t="inlineStr">
+        <is>
+          <t>Janelle</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -4024,7 +4296,9 @@
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B15" s="3" t="n"/>
+      <c r="B15" s="15" t="n">
+        <v>46292</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4157,7 +4431,11 @@
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B11" s="3" t="n"/>
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>Reserve call -&gt; HTTP 200. After: Reserved=2, status=partially_fulfilled, 2 total − 0 in maintenance − 0 reserved elsewhere = 2 available for these dates</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -4165,7 +4443,11 @@
           <t>Pass/Fail/Not Executed/Blocked</t>
         </is>
       </c>
-      <c r="B12" s="3" t="n"/>
+      <c r="B12" s="13" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -4173,7 +4455,11 @@
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B13" s="3" t="n"/>
+      <c r="B13" s="13" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -4181,7 +4467,11 @@
           <t>Executed by</t>
         </is>
       </c>
-      <c r="B14" s="3" t="n"/>
+      <c r="B14" s="13" t="inlineStr">
+        <is>
+          <t>Janelle</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -4189,7 +4479,9 @@
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B15" s="3" t="n"/>
+      <c r="B15" s="15" t="n">
+        <v>46292</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4320,7 +4612,11 @@
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B11" s="3" t="n"/>
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>GET availability as Coordinator -&gt; HTTP 403 ({'error': 'Only Technical Support Staff can check equipment availability'}). POST reserve as Coordinator -&gt; HTTP 403 ({'error': 'Only Technical Support Staff can reserve equipment'}).</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -4328,7 +4624,11 @@
           <t>Pass/Fail/Not Executed/Blocked</t>
         </is>
       </c>
-      <c r="B12" s="3" t="n"/>
+      <c r="B12" s="13" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -4336,7 +4636,11 @@
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B13" s="3" t="n"/>
+      <c r="B13" s="13" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -4344,7 +4648,11 @@
           <t>Executed by</t>
         </is>
       </c>
-      <c r="B14" s="3" t="n"/>
+      <c r="B14" s="13" t="inlineStr">
+        <is>
+          <t>Janelle</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -4352,7 +4660,9 @@
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B15" s="3" t="n"/>
+      <c r="B15" s="15" t="n">
+        <v>46292</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4485,7 +4795,11 @@
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B11" s="3" t="n"/>
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>Portable Stage: HTTP 200, Reserved=2 (reserved). Ring Light: HTTP 200, Reserved=2 (partially_fulfilled). Mobile Charging Cart: HTTP 400 {'error': 'Nothing is available for these dates any more.'}, Reserved stays None.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -4493,7 +4807,11 @@
           <t>Pass/Fail/Not Executed/Blocked</t>
         </is>
       </c>
-      <c r="B12" s="3" t="n"/>
+      <c r="B12" s="13" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -4501,7 +4819,11 @@
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B13" s="3" t="n"/>
+      <c r="B13" s="13" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -4509,7 +4831,11 @@
           <t>Executed by</t>
         </is>
       </c>
-      <c r="B14" s="3" t="n"/>
+      <c r="B14" s="13" t="inlineStr">
+        <is>
+          <t>Janelle</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -4517,7 +4843,9 @@
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B15" s="3" t="n"/>
+      <c r="B15" s="15" t="n">
+        <v>46292</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4650,7 +4978,11 @@
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B11" s="3" t="n"/>
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>After reserving and re-reading (reload): equipment=Portable Stage, Reserved=2, status=reserved.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -4658,7 +4990,11 @@
           <t>Pass/Fail/Not Executed/Blocked</t>
         </is>
       </c>
-      <c r="B12" s="3" t="n"/>
+      <c r="B12" s="13" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -4666,7 +5002,11 @@
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B13" s="3" t="n"/>
+      <c r="B13" s="13" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -4674,7 +5014,11 @@
           <t>Executed by</t>
         </is>
       </c>
-      <c r="B14" s="3" t="n"/>
+      <c r="B14" s="13" t="inlineStr">
+        <is>
+          <t>Janelle</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -4682,7 +5026,9 @@
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B15" s="3" t="n"/>
+      <c r="B15" s="15" t="n">
+        <v>46292</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4815,7 +5161,11 @@
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B11" s="3" t="n"/>
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>Requested 5, available 6 before reserving. After: Reserved=5 (not 6), status=reserved.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -4823,7 +5173,11 @@
           <t>Pass/Fail/Not Executed/Blocked</t>
         </is>
       </c>
-      <c r="B12" s="3" t="n"/>
+      <c r="B12" s="13" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -4831,7 +5185,11 @@
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B13" s="3" t="n"/>
+      <c r="B13" s="13" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -4839,7 +5197,11 @@
           <t>Executed by</t>
         </is>
       </c>
-      <c r="B14" s="3" t="n"/>
+      <c r="B14" s="13" t="inlineStr">
+        <is>
+          <t>Janelle</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -4847,7 +5209,9 @@
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B15" s="3" t="n"/>
+      <c r="B15" s="15" t="n">
+        <v>46292</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4981,7 +5345,11 @@
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B11" s="3" t="n"/>
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>Harvest Fair after reserving: Reserved=2. Summer Fair (unrelated date): Reserved=None, status=under_review.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -4989,7 +5357,11 @@
           <t>Pass/Fail/Not Executed/Blocked</t>
         </is>
       </c>
-      <c r="B12" s="3" t="n"/>
+      <c r="B12" s="13" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -4997,7 +5369,11 @@
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B13" s="3" t="n"/>
+      <c r="B13" s="13" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -5005,7 +5381,11 @@
           <t>Executed by</t>
         </is>
       </c>
-      <c r="B14" s="3" t="n"/>
+      <c r="B14" s="13" t="inlineStr">
+        <is>
+          <t>Janelle</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -5013,7 +5393,9 @@
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B15" s="3" t="n"/>
+      <c r="B15" s="15" t="n">
+        <v>46292</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
SPM-49: confirm a saved reservation; no Reserve button on closed events
- After Reserve succeeds, the line now says "Reservation saved: N reserved."
  (kept across the reload that follows). SPM-49-TC01/TC02 expect a
  confirmation; the page previously only refreshed the numbers.
- A cancelled, postponed, rejected or completed event no longer offers the
  Reserve button; the page says why instead ("This event is cancelled —
  equipment can no longer be reserved."). Before, the button showed and only
  the click was refused (SPM-49-TC18).
- The rule lives in one place, eventAllowsReserving() and
  reservingClosedMessage() in equipmentAvailability.ts, used by both the page
  and the Reserve route, so they cannot disagree. The route's behaviour and
  message are unchanged.
- SPM-49-TC01, TC02 and TC18 expected results updated to the exact wording.
</commit_message>
<xml_diff>
--- a/docs/test-cases/SPM-49_Test_Cases.xlsx
+++ b/docs/test-cases/SPM-49_Test_Cases.xlsx
@@ -3473,8 +3473,8 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>No Reserve button is offered, or clicking it shows the message 'This event is cancelled - equipment can no longer be reserved.' and nothing is reserved.
-The Reserved box stays empty.</t>
+          <t>No Reserve button is offered on the Portable Stage line, and the page shows the message 'This event is cancelled — equipment can no longer be reserved.'
+Nothing is reserved: the Reserved box stays empty.</t>
         </is>
       </c>
     </row>
@@ -4205,7 +4205,7 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>A confirmation that the reservation was saved is shown.
+          <t>The message 'Reservation saved: 3 reserved.' appears on the Portable Stage line.
 The Reserved box on the Portable Stage line shows 3.
 The request status chip shows 'Reserved'.</t>
         </is>
@@ -4388,7 +4388,7 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>A confirmation that the reservation was saved is shown.
+          <t>The message 'Reservation saved: 2 reserved.' appears on the Ring Light line.
 The Reserved box on the Ring Light line shows 2 - the smaller of requested (4) and available (2), never more than either.
 The request status chip shows 'Partially fulfilled'.</t>
         </is>

</xml_diff>